<commit_message>
fix: autofit pads text as Excel does, so column widths and wrapping match Excel's padding (#789)
Measured in Excel 16.0 at 120 DPI over COM: for text W px wide, the autofit width is W + 2*ceil(cellMdw/4) + 1 + max(2, floor(W / (4*mdw))), where mdw is the column's (first font's) digit width. With GDI text widths this gave Excel's width to the pixel for 108 strings in nine fonts and sizes, and for runs of 1 to 120 glyphs. Wrapping uses the same rule. XLibur padded 3 % of the width plus MDW/4 on each side.

The rest of the difference is text measurement (Excel uses GDI hinted advances at a whole-pixel em) and the row line pitch; both are documented in docs/autofit-vs-excel.md and left as they are. FirstFontDigitWidthTests now checks widths within 3.5 % and heights within 5 % (was 10 %). Example reference files are updated for the new column widths only.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Loading/ChangingBasicTable.xlsx
+++ b/XLibur.Tests/Resource/Examples/Loading/ChangingBasicTable.xlsx
@@ -721,11 +721,11 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9.140625"/>
-    <x:col min="2" max="2" width="7.424911" customWidth="1"/>
-    <x:col min="3" max="3" width="8.567768" customWidth="1"/>
-    <x:col min="4" max="4" width="8.139196" customWidth="1"/>
-    <x:col min="5" max="5" width="11.424911" customWidth="1"/>
-    <x:col min="6" max="6" width="15.424911" customWidth="1"/>
+    <x:col min="2" max="2" width="7.139196" customWidth="1"/>
+    <x:col min="3" max="3" width="8.282054" customWidth="1"/>
+    <x:col min="4" max="4" width="7.853482" customWidth="1"/>
+    <x:col min="5" max="5" width="11.139196" customWidth="1"/>
+    <x:col min="6" max="6" width="14.996339" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2" spans="1:6">

</xml_diff>